<commit_message>
chore: persist Round 1 review data to xlsx and restore comments JSON
- WIP_NFL_Survey_v0.xlsx: Round 1 review flags and comments written to
  columns 13-14 ("Review Comment (2026-03-30 R1)", "Review Flag (2026-03-30 R1)")
- nfl_review_comments.json: R1 data restored after accidental test clear

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working/survey/WIP_NFL_Survey_v0.xlsx
+++ b/working/survey/WIP_NFL_Survey_v0.xlsx
@@ -1368,12 +1368,12 @@
       </c>
       <c r="M1" s="11" t="inlineStr">
         <is>
-          <t>Review Comment</t>
+          <t>Review Comment (2026-03-30 R1)</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Review Flag</t>
+          <t>Review Flag (2026-03-30 R1)</t>
         </is>
       </c>
     </row>
@@ -1453,11 +1453,7 @@
         </is>
       </c>
       <c r="L3" s="13" t="n"/>
-      <c r="M3" s="13" t="inlineStr">
-        <is>
-          <t>NFC - Please review answers to make sure that answer "buckets" sizing is correct for NFL Stadiums (C should be avg /reasonable/ passable metric)</t>
-        </is>
-      </c>
+      <c r="M3" s="13" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>revise</t>
@@ -3211,11 +3207,7 @@
         </is>
       </c>
       <c r="L31" s="13" t="n"/>
-      <c r="M31" s="13" t="inlineStr">
-        <is>
-          <t>MARKED FOR DROP — reviewer confirmed not needed in final survey. Remove after Vik review.</t>
-        </is>
-      </c>
+      <c r="M31" s="13" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
           <t>drop</t>
@@ -3279,11 +3271,7 @@
         </is>
       </c>
       <c r="L32" s="13" t="n"/>
-      <c r="M32" s="13" t="inlineStr">
-        <is>
-          <t>MARKED FOR DROP — reviewer confirmed not needed in final survey. Remove after Vik review.</t>
-        </is>
-      </c>
+      <c r="M32" s="13" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>drop</t>
@@ -3349,7 +3337,7 @@
       <c r="L33" s="13" t="n"/>
       <c r="M33" s="13" t="inlineStr">
         <is>
-          <t>MARKED FOR DROP — reviewer confirmed not needed in final survey. Remove after Vik review.</t>
+          <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -4039,7 +4027,7 @@
       <c r="L45" s="13" t="n"/>
       <c r="M45" s="13" t="inlineStr">
         <is>
-          <t>MARKED FOR DROP — reviewer confirmed not needed in final survey. Remove after Vik review.</t>
+          <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -4472,6 +4460,7 @@
           <t>This is a useful use case, but how does that relate to evaluating the stadium infra?</t>
         </is>
       </c>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54" ht="99.95" customHeight="1">
       <c r="A54" s="19" t="inlineStr">
@@ -4728,9 +4717,10 @@
       <c r="L57" s="13" t="n"/>
       <c r="M57" s="13" t="inlineStr">
         <is>
-          <t>MARKED FOR DROP — reviewer confirmed not needed in final survey. Remove after Vik review.</t>
-        </is>
-      </c>
+          <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
survey: reset review comments for Round 2 and update xlsx
Round 1 NFC comments exported to xlsx (export_count 3). Comments and flags
cleared for a fresh Round 2 review pass.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working/survey/WIP_NFL_Survey_v0.xlsx
+++ b/working/survey/WIP_NFL_Survey_v0.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="1" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3000" yWindow="3000" windowWidth="14400" windowHeight="8170" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Layer Definitions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined Survey Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tech Layer Definitions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Combined Survey Questions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -1288,7 +1288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N57"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1376,6 +1376,26 @@
           <t>Review Flag (2026-03-30 R1)</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Review Comment (2026-03-31 R2)</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Review Flag (2026-03-31 R2)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Review Comment (2026-03-31 R3)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Review Flag (2026-03-31 R3)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15.95" customHeight="1" thickBot="1">
       <c r="A2" s="27" t="inlineStr">
@@ -1459,6 +1479,21 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>We should probably think if we can do some sort of adaptive views here.  As the teams won't know this metric, they will only know their total AP count.  Then we'll have to divide that by capacity to get the accurate count.  Then we can reference phase 1 metric for poor, ok, great, etc</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="99.95" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -1523,6 +1558,17 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="87.59999999999999" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
@@ -1587,6 +1633,21 @@
         </is>
       </c>
       <c r="N5" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>They may not have this data as it's not something they are regularly tracking</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>revise</t>
         </is>
@@ -1655,6 +1716,18 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>SHould we consider 4g vs 5g  (we would likely have to split this question out)</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7" ht="87.59999999999999" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -1719,6 +1792,21 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>I don't think private networks are much of a factor in stadiums, unless the opps folks get a private APN or something</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="99.95" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -1787,6 +1875,26 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>NFC - Please review answers to make sure that answer "buckets" sizing is correct for NFL Stadiums (C should be avg /reasonable/ passable metric)</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>this should be a 1 shot question, circuit size: dual 40gb, etc.</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="87.59999999999999" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
@@ -1855,6 +1963,26 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>NFC - Please develop a questions and the rationalized scoring for us and present it for review - (Please review answers to make sure that answer "buckets" sizing is correct for NFL Stadiums (C should be avg /reasonable/ passable metric))</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>they have failover to a backup circuit typically</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="99.95" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -1921,6 +2049,26 @@
       <c r="N10" t="inlineStr">
         <is>
           <t>split</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFC - This question seems like its mixing service quality and cyber security. I also think we need to tighten this question and potentially separate into 2 </t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>getting in the weeds for a cio level discussion, may need to bring up a few levels.</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>revise</t>
         </is>
       </c>
     </row>
@@ -1987,6 +2135,21 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">they most likely don't, "clubs" may have a team of 4-5 total for IT.  1) if it's their network its probably minimal, 2) its likely a managed service from carrier/telco </t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="99.95" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -2051,6 +2214,21 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>why does this matter?  They're gonna have no idea.  Probably created when built or renovated.</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>drop</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="87.59999999999999" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -2115,6 +2293,26 @@
         </is>
       </c>
       <c r="N13" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NFC - We need to rethink how we are asking this question. - think through how team provide a consitant user experience for fans on the wifi? How do was ask that question(s)? How do the prioritieze traffic? </t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Too vague, they're not going to do anything.  You build the network, you tune it for a month.  Then you manage code releases, flappy APs, etc.  Outside of the odd upgrade.</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t>revise</t>
         </is>
@@ -2183,6 +2381,26 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Density footprint on seats my be a repeat / we should consider merging</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>they aren't going to know, it should be baseline 100% coverage, unless offsite parking or something random.</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>drop</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="99.95" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
@@ -2247,6 +2465,26 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>We should consider merging with question 9.</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>its going to be an NMS report, they aren't caring realtime unless there's an outage.</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="99.95" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
@@ -2311,6 +2549,26 @@
         </is>
       </c>
       <c r="N16" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>NFC - We need to refine the response options. this is more of question of how uniform your infrastructure is (have you piece-mealed stuff together over time, or have you designed it with consistent hardware for scalability?)</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>This question feels like AI wrote it, the answers make sense but we need to augment the question phrasing.</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
         <is>
           <t>revise</t>
         </is>
@@ -2413,6 +2671,17 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="99.95" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
@@ -2477,6 +2746,17 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="99.95" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -2545,6 +2825,18 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>NFC - Get rid of caution (this question is good)</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22" ht="99.95" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
@@ -2613,6 +2905,27 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>NFC - Question should be frame more along the lines of do you leverage realtime streaming capabilities enhance fan experience and drive operations. We want to make sure the question/ answer measure streaming capability maturity</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">need some simple examples added to help frame the question
+</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="99.95" customHeight="1">
       <c r="A23" s="19" t="inlineStr">
@@ -2681,6 +2994,26 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>NFC - The point of view should be that they are somewhere along the maturity ladder already - answer c is the ground floor, how can we frame the questions different if we assume that c is a min standard</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>How are APIs relevant to fan experience?</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="87.59999999999999" customHeight="1">
       <c r="A24" s="19" t="inlineStr">
@@ -2749,6 +3082,26 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>NFC - This question is a bit convoluted and I think we need to simplify it a little bit. That being said it is a good measure of maturity. we need to make sure this scoring logic is tighter with no holes. also if we are multi selectic what happens if user select mono and others?</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>seems like a reprint of an infra question</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="99.95" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
@@ -2815,6 +3168,27 @@
       <c r="N25" t="inlineStr">
         <is>
           <t>revise</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>NFC - please draft the possible responses to this question. We want them to be able to select all the identify access management capabilities that they have. The more the have the higher the score</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Maybe simplify the responses, that's alot
+</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -2881,6 +3255,21 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>another reprint answer, any opps/performance stuff should be rolled into a single question that frames across all domains.</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="99.95" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
@@ -2945,6 +3334,21 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>this is called DIGITAL SIGNAGE in this space.  Update the name and remove the e.g.</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="87.59999999999999" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
@@ -3013,6 +3417,26 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>NFC - Please review answers to make sure that answer "buckets" sizing is correct for NFL Stadiums (C should be avg /reasonable/ passable metric)</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>remove 10k seats and just ask for raw count, like the AP question we can backdoor the metric based on capacity</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="87.59999999999999" customHeight="1">
       <c r="A29" s="19" t="inlineStr">
@@ -3081,6 +3505,26 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>NFC - Please review answers to make sure that answer "buckets" sizing is correct for NFL Stadiums (C should be avg /reasonable/ passable metric)</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>think about all security related tech, biometrics, clear pass, etc.</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="112.5" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
@@ -3145,6 +3589,26 @@
         </is>
       </c>
       <c r="N30" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>NFC - do we need Ask this differently? Maybe more like what are you are running on the edge - CDN, ticketing, etc? this would likely be a select all that apply type of question. give me some feedback</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>simplify response and so what of the question</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
         <is>
           <t>revise</t>
         </is>
@@ -3213,6 +3677,21 @@
           <t>drop</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>drop</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>not sure about this one, needs to be locked into scope/objective.</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="99.95" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
@@ -3277,6 +3756,21 @@
           <t>drop</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>drop</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>odd question given the rest of the theme</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="99.95" customHeight="1">
       <c r="A33" s="19" t="inlineStr">
@@ -3343,6 +3837,26 @@
       <c r="N33" t="inlineStr">
         <is>
           <t>drop</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>drop</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>this is something they could use to kick the can on future enhancements and falsely increase their present score.</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>revise</t>
         </is>
       </c>
     </row>
@@ -3443,6 +3957,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37" ht="87.59999999999999" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
@@ -3511,6 +4032,18 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>NFC - This method of scoring is good provided that using more of them at the same time is better, is this the case? Or do we need to ask this questions differnt?</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38" ht="99.95" customHeight="1">
       <c r="A38" s="19" t="inlineStr">
@@ -3579,6 +4112,18 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>NFC - Why would using more POS systems lead to a better score? Having more would likely be a bad thing. This question should be more about how wide spread POS systems are, i.e can I pay for things from my seat, etc., need to make sure scoring is tight</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39" ht="99.95" customHeight="1">
       <c r="A39" s="19" t="inlineStr">
@@ -3643,6 +4188,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40" ht="99.95" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
@@ -3707,6 +4259,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41" ht="87.59999999999999" customHeight="1">
       <c r="A41" s="19" t="inlineStr">
@@ -3771,6 +4330,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42" ht="99.95" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
@@ -3835,6 +4401,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43" ht="99.95" customHeight="1">
       <c r="A43" s="19" t="inlineStr">
@@ -3899,6 +4472,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44" ht="99.95" customHeight="1">
       <c r="A44" s="19" t="inlineStr">
@@ -3967,6 +4547,18 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>NFC - Please review answers to make sure that answer "buckets" sizing is correct for Stadiums/venues (C should be avg /reasonable/ passable metric)</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45" ht="87.59999999999999" customHeight="1">
       <c r="A45" s="19" t="inlineStr">
@@ -4035,6 +4627,18 @@
           <t>drop</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>drop</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46" ht="9.949999999999999" customHeight="1">
       <c r="A46" s="14" t="n"/>
@@ -4133,6 +4737,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
     </row>
     <row r="49" ht="75" customHeight="1">
       <c r="A49" s="19" t="inlineStr">
@@ -4197,6 +4808,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr"/>
+      <c r="R49" t="inlineStr"/>
     </row>
     <row r="50" ht="75" customHeight="1">
       <c r="A50" s="19" t="inlineStr">
@@ -4265,6 +4883,18 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>NFC - question should be more along the lines of which of the Computer vision do you use during game day</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr"/>
+      <c r="R50" t="inlineStr"/>
     </row>
     <row r="51" ht="75" customHeight="1">
       <c r="A51" s="19" t="inlineStr">
@@ -4329,6 +4959,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="inlineStr"/>
     </row>
     <row r="52" ht="87.59999999999999" customHeight="1">
       <c r="A52" s="19" t="inlineStr">
@@ -4397,6 +5034,18 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>NFC - question should be more along the lines of which of the Gen AI do you use during game day</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q52" t="inlineStr"/>
+      <c r="R52" t="inlineStr"/>
     </row>
     <row r="53" ht="99.95" customHeight="1">
       <c r="A53" s="19" t="inlineStr">
@@ -4460,7 +5109,13 @@
           <t>This is a useful use case, but how does that relate to evaluating the stadium infra?</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>This is a useful use case, but how does that relate to evaluating the stadium infra?</t>
+        </is>
+      </c>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
     </row>
     <row r="54" ht="99.95" customHeight="1">
       <c r="A54" s="19" t="inlineStr">
@@ -4529,6 +5184,18 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>NFC - Can we be more detail/ tighter/ descriptive with our answers? We are trying to ask if they have an understanding ofwhere they are going and the investment (capital and time) to get there?</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>revise</t>
+        </is>
+      </c>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55" ht="99.95" customHeight="1">
       <c r="A55" s="19" t="inlineStr">
@@ -4593,6 +5260,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56" ht="99.95" customHeight="1">
       <c r="A56" s="19" t="inlineStr">
@@ -4657,6 +5331,13 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57" ht="87.59999999999999" customHeight="1">
       <c r="A57" s="19" t="inlineStr">
@@ -4720,7 +5401,13 @@
           <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
+        </is>
+      </c>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
fix: restore John's R2/R3 review comments to xlsx; add history view to dashboard
Recovers cols 15-18 from John's branch that were incorrectly removed during
cleanup. R2 = RT3 review comments, R3 = John Sheerin's review comments.
Dashboard Question Review tab now surfaces all 3 rounds (R1/R2/R3) inline
on each question card. /review redirects to dashboard — single review UI.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working/survey/WIP_NFL_Survey_v0.xlsx
+++ b/working/survey/WIP_NFL_Survey_v0.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="1" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3000" yWindow="3000" windowWidth="14400" windowHeight="8170" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tech Layer Definitions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Combined Survey Questions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tech Layer Definitions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined Survey Questions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -1288,7 +1288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:U57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1396,6 +1396,21 @@
           <t>Review Flag (2026-03-31 R3)</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Comment - QA Test (2026-03-31)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Comment - QA Test (2026-03-31)</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Comment - QA Test (2026-03-31)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15.95" customHeight="1" thickBot="1">
       <c r="A2" s="27" t="inlineStr">
@@ -1563,7 +1578,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
           <t>ok</t>
@@ -1726,8 +1740,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7" ht="87.59999999999999" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -2676,7 +2688,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr">
         <is>
           <t>ok</t>
@@ -2751,7 +2762,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr">
         <is>
           <t>ok</t>
@@ -2835,8 +2845,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22" ht="99.95" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
@@ -3962,8 +3970,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37" ht="87.59999999999999" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
@@ -4042,8 +4048,6 @@
           <t>revise</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38" ht="99.95" customHeight="1">
       <c r="A38" s="19" t="inlineStr">
@@ -4122,8 +4126,6 @@
           <t>revise</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39" ht="99.95" customHeight="1">
       <c r="A39" s="19" t="inlineStr">
@@ -4193,8 +4195,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
     </row>
     <row r="40" ht="99.95" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
@@ -4264,8 +4264,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
     </row>
     <row r="41" ht="87.59999999999999" customHeight="1">
       <c r="A41" s="19" t="inlineStr">
@@ -4335,8 +4333,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
     </row>
     <row r="42" ht="99.95" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
@@ -4406,8 +4402,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43" ht="99.95" customHeight="1">
       <c r="A43" s="19" t="inlineStr">
@@ -4477,8 +4471,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44" ht="99.95" customHeight="1">
       <c r="A44" s="19" t="inlineStr">
@@ -4557,8 +4549,6 @@
           <t>revise</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45" ht="87.59999999999999" customHeight="1">
       <c r="A45" s="19" t="inlineStr">
@@ -4637,8 +4627,6 @@
           <t>drop</t>
         </is>
       </c>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46" ht="9.949999999999999" customHeight="1">
       <c r="A46" s="14" t="n"/>
@@ -4742,8 +4730,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
     </row>
     <row r="49" ht="75" customHeight="1">
       <c r="A49" s="19" t="inlineStr">
@@ -4813,8 +4799,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
     </row>
     <row r="50" ht="75" customHeight="1">
       <c r="A50" s="19" t="inlineStr">
@@ -4893,8 +4877,6 @@
           <t>revise</t>
         </is>
       </c>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
     </row>
     <row r="51" ht="75" customHeight="1">
       <c r="A51" s="19" t="inlineStr">
@@ -4964,8 +4946,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
     </row>
     <row r="52" ht="87.59999999999999" customHeight="1">
       <c r="A52" s="19" t="inlineStr">
@@ -5044,8 +5024,6 @@
           <t>revise</t>
         </is>
       </c>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
     </row>
     <row r="53" ht="99.95" customHeight="1">
       <c r="A53" s="19" t="inlineStr">
@@ -5114,8 +5092,6 @@
           <t>This is a useful use case, but how does that relate to evaluating the stadium infra?</t>
         </is>
       </c>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
     </row>
     <row r="54" ht="99.95" customHeight="1">
       <c r="A54" s="19" t="inlineStr">
@@ -5194,8 +5170,6 @@
           <t>revise</t>
         </is>
       </c>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
     </row>
     <row r="55" ht="99.95" customHeight="1">
       <c r="A55" s="19" t="inlineStr">
@@ -5265,8 +5239,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
     </row>
     <row r="56" ht="99.95" customHeight="1">
       <c r="A56" s="19" t="inlineStr">
@@ -5336,8 +5308,6 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57" ht="87.59999999999999" customHeight="1">
       <c r="A57" s="19" t="inlineStr">
@@ -5406,8 +5376,6 @@
           <t>This may be a question ask during workshops so that we can track the planned development, but not needed in the final survey</t>
         </is>
       </c>
-      <c r="Q57" t="inlineStr"/>
-      <c r="R57" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
sync: NFL survey review session Apr 2 — reviewer metadata + timestamp reset
Updated nfl_review_comments.json: reviewer tagged as "Team - RT3, Kieran, Vik",
last_updated/last_reset bumped to 2026-04-02, export_count 3. WIP_NFL_Survey_v0.xlsx
updated in sync.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/working/survey/WIP_NFL_Survey_v0.xlsx
+++ b/working/survey/WIP_NFL_Survey_v0.xlsx
@@ -1288,7 +1288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U57"/>
+  <dimension ref="A1:V57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.45"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1411,6 +1411,11 @@
           <t>Comment - QA Test (2026-03-31)</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Comment - Team - RT3, Kieran, Vik (2026-04-02)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15.95" customHeight="1" thickBot="1">
       <c r="A2" s="27" t="inlineStr">
@@ -1509,6 +1514,11 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>[OK]</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="99.95" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -1583,6 +1593,11 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>[OK]</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="87.59999999999999" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
@@ -1664,6 +1679,11 @@
       <c r="R5" t="inlineStr">
         <is>
           <t>revise</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>[REVISE] Come back to - may be too specific of a question, play with wording</t>
         </is>
       </c>
     </row>
@@ -1740,6 +1760,11 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>[REVISE] Change wording "activiely" - don't include CBRS</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="87.59999999999999" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -1819,6 +1844,11 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>[REVISE] We need better phrasing of the questions. - we need to ask the question in a better fashion, should be just about the level of capabilities. - we need to make sure that their are no overlapping questions</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="99.95" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -1905,6 +1935,11 @@
       <c r="R8" t="inlineStr">
         <is>
           <t>revise</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>[OK]</t>
         </is>
       </c>
     </row>
@@ -2162,6 +2197,11 @@
           <t>revise</t>
         </is>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>[REVISE] The real question is how much control you have over network ops - then lay out control levers (what cabilities do t they have with their current structure)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="99.95" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -2583,6 +2623,11 @@
       <c r="R16" t="inlineStr">
         <is>
           <t>revise</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>[REVISE] Tighten question phrasing</t>
         </is>
       </c>
     </row>
@@ -2693,6 +2738,11 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>[REVISE] Describe your</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="99.95" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
@@ -2767,6 +2817,11 @@
           <t>ok</t>
         </is>
       </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>[REVISE] We shoudl be asking more describe how they utilize edge compute - make the assumption that they have it</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="99.95" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -2843,6 +2898,11 @@
       <c r="P21" t="inlineStr">
         <is>
           <t>ok</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>[REVISE] rethink/rephrase question - how do they secure and store data (do they have on-prem data center) can we sqeeze into the data infra question.</t>
         </is>
       </c>
     </row>

</xml_diff>